<commit_message>
Add some chipsat stuff
</commit_message>
<xml_diff>
--- a/analyses/Misc_Spreadsheet.xlsx
+++ b/analyses/Misc_Spreadsheet.xlsx
@@ -1,26 +1,274 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\konstantinos.kanavou\Documents\git\phd-thesis\analyses\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{FAFCA73A-1CD7-4AA7-A707-F07C51B69787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Chipsat-1 Work" sheetId="1" r:id="rId1"/>
+    <sheet name="ChipSat-1 Cost" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
+  <si>
+    <t>ChipSat-1 Person Hours</t>
+  </si>
+  <si>
+    <t>Hours</t>
+  </si>
+  <si>
+    <t>Sample of initial data: 2022-11</t>
+  </si>
+  <si>
+    <t>Systems Engineering (K)</t>
+  </si>
+  <si>
+    <t>Project Management (O)</t>
+  </si>
+  <si>
+    <t>Orbital Analysis</t>
+  </si>
+  <si>
+    <t>Antenna Simulation</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>Test Campaign QM</t>
+  </si>
+  <si>
+    <t>Test Campaign FM</t>
+  </si>
+  <si>
+    <t>Test Campaign Antenna</t>
+  </si>
+  <si>
+    <t>Antenna Testing E/M</t>
+  </si>
+  <si>
+    <t>Person Months</t>
+  </si>
+  <si>
+    <t>Scenario 0: Actual</t>
+  </si>
+  <si>
+    <t>Prototyping (K)</t>
+  </si>
+  <si>
+    <t>Integration (K)</t>
+  </si>
+  <si>
+    <t>Software Development (K)</t>
+  </si>
+  <si>
+    <t>Processed data</t>
+  </si>
+  <si>
+    <t>Cost driver</t>
+  </si>
+  <si>
+    <t>Cost (EUR)</t>
+  </si>
+  <si>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>Percentage of total costs</t>
+  </si>
+  <si>
+    <t>Breadboard model</t>
+  </si>
+  <si>
+    <t>Components purchase</t>
+  </si>
+  <si>
+    <t>0,6</t>
+  </si>
+  <si>
+    <t>Structural model (SM)</t>
+  </si>
+  <si>
+    <t>The ChipSat-1 SM was built with an empty PCB and the antennas with their deployment mechanism</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>SM testing</t>
+  </si>
+  <si>
+    <t>Costs of vibration testing (detailed in Table 4)</t>
+  </si>
+  <si>
+    <t>7,3</t>
+  </si>
+  <si>
+    <t>Interface bracket for SM testing and adapters for test platform</t>
+  </si>
+  <si>
+    <t>One aluminum interface bracket and two vibration test adapters (vertical + horizontal)</t>
+  </si>
+  <si>
+    <t>8,9</t>
+  </si>
+  <si>
+    <t>Costs from components purchasing, manufacturing, and assembly with subcontractor</t>
+  </si>
+  <si>
+    <t>14,9</t>
+  </si>
+  <si>
+    <t>16,3</t>
+  </si>
+  <si>
+    <t>ChipSat-1 qualification</t>
+  </si>
+  <si>
+    <t>Costs of qualification testing, random vibration + thermal vacuum and thermal cycling (detailed in Table 4)</t>
+  </si>
+  <si>
+    <t>15,2</t>
+  </si>
+  <si>
+    <t>ChipSat-1 acceptance</t>
+  </si>
+  <si>
+    <t>Costs of acceptance testing, random vibrations (detailed in Table 4)</t>
+  </si>
+  <si>
+    <t>Interface bracket with payload and qualification and acceptance test adapters</t>
+  </si>
+  <si>
+    <t>Two sets of interface brackets and qualification and acceptance tests adapters were manufactured due to last minute interface requirements change</t>
+  </si>
+  <si>
+    <t>(580EUR spent on brackets and adapters that were obsolete after late design changes)</t>
+  </si>
+  <si>
+    <t>21,3</t>
+  </si>
+  <si>
+    <t>Total costs</t>
+  </si>
+  <si>
+    <t>Interface bracket with payload and qualification and acceptance test adapters
+Obsolete brackets and adapters after late design changes</t>
+  </si>
+  <si>
+    <t>Iter</t>
+  </si>
+  <si>
+    <t>1,3</t>
+  </si>
+  <si>
+    <t>4,5</t>
+  </si>
+  <si>
+    <t>EM Manufacturing + Components</t>
+  </si>
+  <si>
+    <t>QM and FM Manufacturing + Components</t>
+  </si>
+  <si>
+    <t>CRITERION</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>BM/EM model yes/no</t>
+  </si>
+  <si>
+    <t>Extra time spent in design</t>
+  </si>
+  <si>
+    <t>Single slice yes/no</t>
+  </si>
+  <si>
+    <t>Analysis instead of test yes/no</t>
+  </si>
+  <si>
+    <t>Constants</t>
+  </si>
+  <si>
+    <t>Salary/Hour</t>
+  </si>
+  <si>
+    <t>Init. Redesign Chance</t>
+  </si>
+  <si>
+    <t>Cumul. Redesign Chance</t>
+  </si>
+  <si>
+    <t>Cost of Redesign</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +276,50 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -45,14 +327,142 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -66,6 +476,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>476249</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>229279</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>240232</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>201239</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C1C6627-A49C-AD5F-5FA1-F187D7478EE3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12125324" y="619804"/>
+          <a:ext cx="10127183" cy="5829835"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -330,10 +789,635 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>48</v>
+      </c>
+      <c r="D4">
+        <f>B4</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>112</v>
+      </c>
+      <c r="D9">
+        <f>B9</f>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10">
+        <f>B10</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11">
+        <f>B11</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14">
+        <v>12</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15">
+        <f>3*8</f>
+        <v>24</v>
+      </c>
+      <c r="D15">
+        <f>B15</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <f>3*8</f>
+        <v>24</v>
+      </c>
+      <c r="D16">
+        <f>B16</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="2" cm="1">
+        <f t="array" ref="B19">SUM(B3:B18/152)</f>
+        <v>3.1447368421052633</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D23" s="3"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="16">
+        <v>133</v>
+      </c>
+      <c r="D25" s="17">
+        <v>0.25</v>
+      </c>
+      <c r="F25" s="17">
+        <v>0.25</v>
+      </c>
+      <c r="H25">
+        <f>2690+75*B25</f>
+        <v>12665</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" t="s">
+        <v>54</v>
+      </c>
+      <c r="D28" t="s">
+        <v>55</v>
+      </c>
+      <c r="E28" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" s="15">
+        <f>-450-1270</f>
+        <v>-1720</v>
+      </c>
+      <c r="D29" s="15">
+        <f>-75</f>
+        <v>-75</v>
+      </c>
+      <c r="E29" s="15">
+        <v>3</v>
+      </c>
+      <c r="G29" s="15">
+        <f>C29+$B$25*D29+($D$25+E29*$F$25)*$H$25</f>
+        <v>970</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30" s="15">
+        <v>0</v>
+      </c>
+      <c r="D30" s="15">
+        <v>75</v>
+      </c>
+      <c r="E30" s="15">
+        <v>-2</v>
+      </c>
+      <c r="G30" s="15">
+        <f t="shared" ref="G30:G32" si="0">C30+$B$25*D30+($D$25+E30*$F$25)*$H$25</f>
+        <v>6808.75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31">
+        <v>3</v>
+      </c>
+      <c r="C31" s="15">
+        <f>120</f>
+        <v>120</v>
+      </c>
+      <c r="D31" s="15">
+        <v>75</v>
+      </c>
+      <c r="E31" s="15">
+        <f>-1</f>
+        <v>-1</v>
+      </c>
+      <c r="G31" s="15">
+        <f t="shared" si="0"/>
+        <v>10095</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32">
+        <v>4</v>
+      </c>
+      <c r="C32" s="15">
+        <f>-630-760</f>
+        <v>-1390</v>
+      </c>
+      <c r="D32" s="15">
+        <f>48+132-12-48</f>
+        <v>120</v>
+      </c>
+      <c r="E32" s="15">
+        <v>1</v>
+      </c>
+      <c r="G32" s="15">
+        <f t="shared" si="0"/>
+        <v>20902.5</v>
+      </c>
+    </row>
+    <row r="33" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+    </row>
+    <row r="34" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+    </row>
+    <row r="35" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+    </row>
+    <row r="36" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B4:B16">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{3DF8A6F9-E484-4A5A-8595-8DE72EA63AA4}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D16">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFB628"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{3690F3D7-C591-4B98-916A-5B0D8BD1D492}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{3DF8A6F9-E484-4A5A-8595-8DE72EA63AA4}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>B4:B16</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{3690F3D7-C591-4B98-916A-5B0D8BD1D492}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D4:D16</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{158E47E8-D1A2-4478-949E-7BB55C35260F}">
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr defaultRowHeight="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="62.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5703125" customWidth="1"/>
+    <col min="4" max="4" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="7">
+        <f>334+120</f>
+        <v>454</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="7">
+        <v>5</v>
+      </c>
+      <c r="C3" s="7">
+        <v>3</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="7">
+        <v>1274</v>
+      </c>
+      <c r="C4" s="7">
+        <v>2</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="7">
+        <v>625</v>
+      </c>
+      <c r="C5" s="7">
+        <v>3</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="7">
+        <v>760</v>
+      </c>
+      <c r="C6" s="7">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="7">
+        <v>1392</v>
+      </c>
+      <c r="C7" s="7">
+        <v>4</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1300</v>
+      </c>
+      <c r="C8" s="7">
+        <v>4</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="7">
+        <v>1300</v>
+      </c>
+      <c r="C9" s="7">
+        <v>5</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="11">
+        <v>580</v>
+      </c>
+      <c r="C10" s="11">
+        <v>3</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+    </row>
+    <row r="11" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="8"/>
+    </row>
+    <row r="12" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="11">
+        <f>1820-580</f>
+        <v>1240</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="12"/>
+    </row>
+    <row r="14" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="7">
+        <f>SUM(B2:B13)</f>
+        <v>8930</v>
+      </c>
+      <c r="C14" s="14"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+    </row>
+    <row r="15" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13"/>
+    </row>
+    <row r="16" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D16">
+        <f>450+1270+5+760+630+1390+580+1240+1300+1300</f>
+        <v>8925</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="C12:C13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Start work on POQUITO
</commit_message>
<xml_diff>
--- a/analyses/Misc_Spreadsheet.xlsx
+++ b/analyses/Misc_Spreadsheet.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\konstantinos.kanavou\Documents\git\phd-thesis\analyses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{FAFCA73A-1CD7-4AA7-A707-F07C51B69787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8076AB45-0C1D-4704-836B-DA5BF8B6839E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="2985" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chipsat-1 Work" sheetId="1" r:id="rId1"/>
-    <sheet name="ChipSat-1 Cost" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
+    <sheet name="ChipSat-1 Cost" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="79">
   <si>
     <t>ChipSat-1 Person Hours</t>
   </si>
@@ -259,6 +259,45 @@
   </si>
   <si>
     <t>Cost of Redesign</t>
+  </si>
+  <si>
+    <t>POQUITO Person hours</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Development Time Driver</t>
+  </si>
+  <si>
+    <t>Time Spent hours</t>
+  </si>
+  <si>
+    <t>Prototyping</t>
+  </si>
+  <si>
+    <t>Integration</t>
+  </si>
+  <si>
+    <t>Software Development</t>
+  </si>
+  <si>
+    <t>Project Management</t>
+  </si>
+  <si>
+    <t>Antenna Testing</t>
+  </si>
+  <si>
+    <t>Test Campaign (Structural Model)</t>
+  </si>
+  <si>
+    <t>Test Campaign (QM)</t>
+  </si>
+  <si>
+    <t>Test Campaign (FM)</t>
+  </si>
+  <si>
+    <t>Total Time</t>
   </si>
 </sst>
 </file>
@@ -417,7 +456,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -445,21 +484,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -973,13 +1018,13 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="16">
+      <c r="B25" s="14">
         <v>133</v>
       </c>
-      <c r="D25" s="17">
+      <c r="D25" s="15">
         <v>0.25</v>
       </c>
-      <c r="F25" s="17">
+      <c r="F25" s="15">
         <v>0.25</v>
       </c>
       <c r="H25">
@@ -1008,18 +1053,18 @@
       <c r="B29">
         <v>1</v>
       </c>
-      <c r="C29" s="15">
+      <c r="C29" s="13">
         <f>-450-1270</f>
         <v>-1720</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="13">
         <f>-75</f>
         <v>-75</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="13">
         <v>3</v>
       </c>
-      <c r="G29" s="15">
+      <c r="G29" s="13">
         <f>C29+$B$25*D29+($D$25+E29*$F$25)*$H$25</f>
         <v>970</v>
       </c>
@@ -1031,16 +1076,16 @@
       <c r="B30">
         <v>2</v>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="13">
         <v>0</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="13">
         <v>75</v>
       </c>
-      <c r="E30" s="15">
+      <c r="E30" s="13">
         <v>-2</v>
       </c>
-      <c r="G30" s="15">
+      <c r="G30" s="13">
         <f t="shared" ref="G30:G32" si="0">C30+$B$25*D30+($D$25+E30*$F$25)*$H$25</f>
         <v>6808.75</v>
       </c>
@@ -1052,18 +1097,18 @@
       <c r="B31">
         <v>3</v>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="13">
         <f>120</f>
         <v>120</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="13">
         <v>75</v>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="13">
         <f>-1</f>
         <v>-1</v>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="13">
         <f t="shared" si="0"/>
         <v>10095</v>
       </c>
@@ -1075,41 +1120,41 @@
       <c r="B32">
         <v>4</v>
       </c>
-      <c r="C32" s="15">
+      <c r="C32" s="13">
         <f>-630-760</f>
         <v>-1390</v>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="13">
         <f>48+132-12-48</f>
         <v>120</v>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="13">
         <v>1</v>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="13">
         <f t="shared" si="0"/>
         <v>20902.5</v>
       </c>
     </row>
     <row r="33" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C33" s="15"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
     </row>
     <row r="34" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C34" s="15"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
     </row>
     <row r="35" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
     </row>
     <row r="36" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B4:B16">
@@ -1174,6 +1219,161 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC0F0396-91EB-4EA5-913D-6AE4021F629A}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18">
+        <v>1</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" s="18">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18">
+        <v>2</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="18">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18">
+        <v>3</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" s="18">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18">
+        <v>4</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="18">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18">
+        <v>5</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18">
+        <v>6</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="18">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18">
+        <v>7</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="18">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18">
+        <v>9</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="18">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18">
+        <v>10</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="18">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18">
+        <v>11</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="18">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18"/>
+      <c r="B14" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C14" s="18">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="18"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="18"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{158E47E8-D1A2-4478-949E-7BB55C35260F}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1340,51 +1540,51 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="16">
         <v>580</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="16">
         <v>3</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
     </row>
     <row r="11" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
       <c r="D11" s="7"/>
       <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="16">
         <f>1820-580</f>
         <v>1240</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="16" t="s">
         <v>50</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="16" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
       <c r="D13" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="12"/>
+      <c r="E13" s="17"/>
     </row>
     <row r="14" spans="1:5" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
@@ -1394,12 +1594,12 @@
         <f>SUM(B2:B13)</f>
         <v>8930</v>
       </c>
-      <c r="C14" s="14"/>
+      <c r="C14" s="12"/>
       <c r="D14" s="10"/>
       <c r="E14" s="10"/>
     </row>
     <row r="15" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="13"/>
+      <c r="A15" s="11"/>
     </row>
     <row r="16" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D16">

</xml_diff>